<commit_message>
📊 Steam 차트 업데이트: 2026-05-17
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -534,7 +534,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -573,7 +573,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -612,7 +612,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -651,7 +651,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -690,7 +690,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -729,7 +729,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -768,7 +768,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -807,7 +807,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -846,7 +846,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -885,7 +885,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -924,7 +924,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -963,7 +963,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1002,7 +1002,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1041,7 +1041,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1080,7 +1080,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1119,7 +1119,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1158,7 +1158,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1197,7 +1197,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1236,7 +1236,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1275,7 +1275,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1314,7 +1314,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1353,7 +1353,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1392,7 +1392,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1431,7 +1431,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1470,7 +1470,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1509,7 +1509,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1548,7 +1548,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1587,7 +1587,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1626,7 +1626,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1665,7 +1665,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1704,7 +1704,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1743,7 +1743,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1782,7 +1782,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1821,7 +1821,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1860,7 +1860,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -1899,7 +1899,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1938,7 +1938,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -1977,7 +1977,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2016,7 +2016,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2055,7 +2055,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2094,7 +2094,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2133,7 +2133,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2172,7 +2172,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2211,7 +2211,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2250,7 +2250,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2289,7 +2289,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2328,7 +2328,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2367,7 +2367,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2406,7 +2406,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2445,7 +2445,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-17</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2507,7 +2507,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-05-16</t>
+          <t>Steam 인기 차트 — 2026-05-17</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3830,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-05-16</t>
+          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-05-17</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3940,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-05-16</t>
+          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-05-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-09-08
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -534,7 +534,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -573,7 +573,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -612,7 +612,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -651,7 +651,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -690,7 +690,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -729,7 +729,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -768,7 +768,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -807,7 +807,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -846,7 +846,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -885,7 +885,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -924,7 +924,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -963,7 +963,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1002,7 +1002,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1041,7 +1041,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1068,10 +1068,10 @@
         <v>127273</v>
       </c>
       <c r="I15" t="n">
-        <v>45800</v>
+        <v>34350</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="K15" t="n">
         <v>45800</v>
@@ -1080,7 +1080,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1119,7 +1119,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1158,7 +1158,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1197,7 +1197,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1224,10 +1224,10 @@
         <v>1373979</v>
       </c>
       <c r="I19" t="n">
-        <v>5500</v>
+        <v>11000</v>
       </c>
       <c r="J19" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
         <v>11000</v>
@@ -1236,7 +1236,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1275,7 +1275,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1314,7 +1314,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1353,7 +1353,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1392,7 +1392,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1431,7 +1431,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1470,7 +1470,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1509,7 +1509,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1548,7 +1548,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1587,7 +1587,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1614,10 +1614,10 @@
         <v>612177</v>
       </c>
       <c r="I29" t="n">
-        <v>10890</v>
+        <v>16500</v>
       </c>
       <c r="J29" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="K29" t="n">
         <v>16500</v>
@@ -1626,7 +1626,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1665,7 +1665,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1692,10 +1692,10 @@
         <v>599805</v>
       </c>
       <c r="I31" t="n">
-        <v>4510</v>
+        <v>20500</v>
       </c>
       <c r="J31" t="n">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="K31" t="n">
         <v>20500</v>
@@ -1704,7 +1704,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1743,7 +1743,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1782,7 +1782,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1821,7 +1821,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1860,7 +1860,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -1899,7 +1899,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1938,7 +1938,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -1977,7 +1977,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2016,7 +2016,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2055,7 +2055,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2094,7 +2094,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2133,7 +2133,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2172,7 +2172,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2211,7 +2211,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2250,7 +2250,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2289,7 +2289,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2328,7 +2328,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2367,7 +2367,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2406,7 +2406,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2445,7 +2445,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2507,7 +2507,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-09-07</t>
+          <t>Steam 인기 차트 — 2026-09-08</t>
         </is>
       </c>
     </row>
@@ -2874,28 +2874,28 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Monster Hunter Wilds</t>
         </is>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" s="4" t="n">
         <v>12494</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" s="4" t="n">
         <v>58.3</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="4" t="n">
         <v>218415</v>
       </c>
-      <c r="F17" t="n">
-        <v>45800</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
+      <c r="F17" s="4" t="n">
+        <v>34350</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="18">
@@ -2974,28 +2974,28 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="n">
+      <c r="A21" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Terraria</t>
         </is>
       </c>
-      <c r="C21" s="4" t="n">
+      <c r="C21" t="n">
         <v>24580</v>
       </c>
-      <c r="D21" s="4" t="n">
+      <c r="D21" t="n">
         <v>97.5</v>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="E21" t="n">
         <v>1409473</v>
       </c>
-      <c r="F21" s="4" t="n">
-        <v>5500</v>
-      </c>
-      <c r="G21" s="4" t="n">
-        <v>50</v>
+      <c r="F21" t="n">
+        <v>11000</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -3224,28 +3224,28 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="n">
+      <c r="A31" t="n">
         <v>28</v>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>ARK: Survival Evolved</t>
         </is>
       </c>
-      <c r="C31" s="4" t="n">
+      <c r="C31" t="n">
         <v>22170</v>
       </c>
-      <c r="D31" s="4" t="n">
+      <c r="D31" t="n">
         <v>83.8</v>
       </c>
-      <c r="E31" s="4" t="n">
+      <c r="E31" t="n">
         <v>730170</v>
       </c>
-      <c r="F31" s="4" t="n">
-        <v>10890</v>
-      </c>
-      <c r="G31" s="4" t="n">
-        <v>34</v>
+      <c r="F31" t="n">
+        <v>16500</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -3274,28 +3274,28 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="n">
+      <c r="A33" t="n">
         <v>30</v>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>The Forest</t>
         </is>
       </c>
-      <c r="C33" s="4" t="n">
+      <c r="C33" t="n">
         <v>2892</v>
       </c>
-      <c r="D33" s="4" t="n">
+      <c r="D33" t="n">
         <v>95.5</v>
       </c>
-      <c r="E33" s="4" t="n">
+      <c r="E33" t="n">
         <v>627791</v>
       </c>
-      <c r="F33" s="4" t="n">
-        <v>4510</v>
-      </c>
-      <c r="G33" s="4" t="n">
-        <v>78</v>
+      <c r="F33" t="n">
+        <v>20500</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -3830,7 +3830,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-09-07</t>
+          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-09-08</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3940,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-09-07</t>
+          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-09-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-09-09
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -534,7 +534,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -573,7 +573,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -612,7 +612,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -651,7 +651,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -678,10 +678,10 @@
         <v>358266</v>
       </c>
       <c r="I5" t="n">
-        <v>22400</v>
+        <v>32000</v>
       </c>
       <c r="J5" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
         <v>32000</v>
@@ -690,7 +690,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -729,7 +729,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -768,7 +768,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -807,7 +807,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -846,7 +846,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -885,7 +885,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -924,7 +924,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -963,7 +963,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1002,7 +1002,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1041,7 +1041,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1080,7 +1080,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1119,7 +1119,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1158,7 +1158,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1197,7 +1197,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1236,7 +1236,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1275,7 +1275,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1314,7 +1314,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1353,7 +1353,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1392,7 +1392,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1431,7 +1431,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1470,7 +1470,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1509,7 +1509,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1548,7 +1548,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1587,7 +1587,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1626,7 +1626,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1665,7 +1665,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1704,7 +1704,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1743,7 +1743,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1782,7 +1782,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1821,7 +1821,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1860,7 +1860,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -1899,7 +1899,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1938,7 +1938,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -1977,7 +1977,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2016,7 +2016,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2055,7 +2055,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2094,7 +2094,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2133,7 +2133,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2172,7 +2172,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2199,10 +2199,10 @@
         <v>643681</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>3300</v>
+        <v>5500</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>5500</v>
@@ -2211,7 +2211,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2250,7 +2250,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2289,7 +2289,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2328,7 +2328,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2367,7 +2367,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2406,7 +2406,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2445,7 +2445,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2507,7 +2507,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-09-08</t>
+          <t>Steam 인기 차트 — 2026-09-09</t>
         </is>
       </c>
     </row>
@@ -2624,28 +2624,28 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n">
+      <c r="A7" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Palworld</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" t="n">
         <v>18028</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" t="n">
         <v>94.09999999999999</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" t="n">
         <v>380709</v>
       </c>
-      <c r="F7" s="4" t="n">
-        <v>22400</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>30</v>
+      <c r="F7" t="n">
+        <v>32000</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -3599,28 +3599,28 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="n">
+      <c r="A46" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>Among Us</t>
         </is>
       </c>
-      <c r="C46" s="4" t="n">
+      <c r="C46" s="2" t="n">
         <v>3832</v>
       </c>
-      <c r="D46" s="4" t="n">
+      <c r="D46" s="2" t="n">
         <v>91.90000000000001</v>
       </c>
-      <c r="E46" s="4" t="n">
+      <c r="E46" s="2" t="n">
         <v>700785</v>
       </c>
-      <c r="F46" s="4" t="n">
-        <v>3300</v>
-      </c>
-      <c r="G46" s="4" t="n">
-        <v>40</v>
+      <c r="F46" s="2" t="n">
+        <v>5500</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -3830,7 +3830,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-09-08</t>
+          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-09-09</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3940,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-09-08</t>
+          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-09-09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-09-10
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -534,7 +534,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -573,7 +573,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -612,7 +612,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -651,7 +651,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -690,7 +690,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -729,7 +729,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -768,7 +768,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -807,7 +807,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -846,7 +846,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -885,7 +885,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -924,7 +924,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -963,7 +963,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1002,7 +1002,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1041,7 +1041,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1080,7 +1080,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1119,7 +1119,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1158,7 +1158,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1197,7 +1197,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1236,7 +1236,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1275,7 +1275,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1314,7 +1314,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1353,7 +1353,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1392,7 +1392,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1431,7 +1431,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1470,7 +1470,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1509,7 +1509,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1548,7 +1548,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1587,7 +1587,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1626,7 +1626,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1665,7 +1665,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1704,7 +1704,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1743,7 +1743,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1782,7 +1782,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1821,7 +1821,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1860,7 +1860,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -1899,7 +1899,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1938,7 +1938,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -1977,7 +1977,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2016,7 +2016,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2055,7 +2055,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2094,7 +2094,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2133,7 +2133,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2172,7 +2172,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2211,7 +2211,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2250,7 +2250,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2289,7 +2289,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2328,7 +2328,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2367,7 +2367,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2406,7 +2406,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2445,7 +2445,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2507,7 +2507,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-09-09</t>
+          <t>Steam 인기 차트 — 2026-09-10</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3830,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-09-09</t>
+          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-09-10</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3940,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-09-09</t>
+          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-09-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-09-11
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -534,7 +534,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -573,7 +573,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -612,7 +612,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -651,7 +651,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -690,7 +690,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -729,7 +729,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -768,7 +768,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -807,7 +807,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -846,7 +846,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -885,7 +885,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -924,7 +924,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -963,7 +963,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1002,7 +1002,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1041,7 +1041,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1080,7 +1080,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1119,7 +1119,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1158,7 +1158,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1197,7 +1197,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1236,7 +1236,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1275,7 +1275,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1314,7 +1314,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1353,7 +1353,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1392,7 +1392,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1431,7 +1431,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1470,7 +1470,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1509,7 +1509,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1548,7 +1548,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1587,7 +1587,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1626,7 +1626,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1665,7 +1665,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1704,7 +1704,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1743,7 +1743,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1782,7 +1782,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1821,7 +1821,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1860,7 +1860,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -1899,7 +1899,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1938,7 +1938,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -1977,7 +1977,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2016,7 +2016,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2055,7 +2055,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2094,7 +2094,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2133,7 +2133,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2172,7 +2172,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2211,7 +2211,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2250,7 +2250,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2277,10 +2277,10 @@
         <v>272900</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>21000</v>
+        <v>5250</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="K46" s="2" t="n">
         <v>21000</v>
@@ -2289,7 +2289,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2328,7 +2328,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2367,7 +2367,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2406,7 +2406,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2445,7 +2445,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2507,7 +2507,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-09-10</t>
+          <t>Steam 인기 차트 — 2026-09-11</t>
         </is>
       </c>
     </row>
@@ -3649,28 +3649,28 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>Borderlands 2</t>
         </is>
       </c>
-      <c r="C48" s="2" t="n">
+      <c r="C48" s="4" t="n">
         <v>8551</v>
       </c>
-      <c r="D48" s="2" t="n">
+      <c r="D48" s="4" t="n">
         <v>92.40000000000001</v>
       </c>
-      <c r="E48" s="2" t="n">
+      <c r="E48" s="4" t="n">
         <v>295218</v>
       </c>
-      <c r="F48" s="2" t="n">
-        <v>21000</v>
-      </c>
-      <c r="G48" s="2" t="n">
-        <v>0</v>
+      <c r="F48" s="4" t="n">
+        <v>5250</v>
+      </c>
+      <c r="G48" s="4" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="49">
@@ -3830,7 +3830,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-09-10</t>
+          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-09-11</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3940,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-09-10</t>
+          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-09-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-09-12
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -534,7 +534,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -573,7 +573,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -612,7 +612,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -651,7 +651,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -690,7 +690,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -729,7 +729,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -768,7 +768,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -807,7 +807,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -846,7 +846,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -885,7 +885,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -924,7 +924,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -963,7 +963,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1002,7 +1002,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1041,7 +1041,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1080,7 +1080,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1119,7 +1119,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1158,7 +1158,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1197,7 +1197,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1236,7 +1236,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1275,7 +1275,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1314,7 +1314,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1353,7 +1353,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1392,7 +1392,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1431,7 +1431,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1470,7 +1470,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1509,7 +1509,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1548,7 +1548,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1587,7 +1587,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1626,7 +1626,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1665,7 +1665,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1704,7 +1704,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1743,7 +1743,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1782,7 +1782,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1821,7 +1821,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1860,7 +1860,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -1899,7 +1899,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1938,7 +1938,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -1977,7 +1977,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2016,7 +2016,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2055,7 +2055,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2094,7 +2094,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2133,7 +2133,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2172,7 +2172,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2211,7 +2211,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2250,7 +2250,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2289,7 +2289,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2328,7 +2328,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2367,7 +2367,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2406,7 +2406,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2445,7 +2445,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2507,7 +2507,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-09-11</t>
+          <t>Steam 인기 차트 — 2026-09-12</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3830,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-09-11</t>
+          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-09-12</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3940,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-09-11</t>
+          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-09-12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Steam 차트 업데이트: 2026-09-13
</commit_message>
<xml_diff>
--- a/steam_chart_tracker.xlsx
+++ b/steam_chart_tracker.xlsx
@@ -534,7 +534,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -573,7 +573,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -612,7 +612,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -651,7 +651,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -690,7 +690,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -729,7 +729,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -768,7 +768,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -807,7 +807,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -846,7 +846,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -885,7 +885,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -924,7 +924,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -963,7 +963,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1002,7 +1002,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1041,7 +1041,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1080,7 +1080,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1119,7 +1119,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1158,7 +1158,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1197,7 +1197,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1236,7 +1236,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -1275,7 +1275,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1314,7 +1314,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -1353,7 +1353,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1392,7 +1392,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -1431,7 +1431,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1470,7 +1470,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -1509,7 +1509,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1536,10 +1536,10 @@
         <v>1071135</v>
       </c>
       <c r="I27" t="n">
-        <v>42000</v>
+        <v>21000</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="K27" t="n">
         <v>42000</v>
@@ -1548,7 +1548,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -1587,7 +1587,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1626,7 +1626,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -1665,7 +1665,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1704,7 +1704,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -1743,7 +1743,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1782,7 +1782,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -1821,7 +1821,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1860,7 +1860,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -1899,7 +1899,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1938,7 +1938,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -1977,7 +1977,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2016,7 +2016,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -2055,7 +2055,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2094,7 +2094,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
@@ -2133,7 +2133,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2172,7 +2172,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -2211,7 +2211,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2250,7 +2250,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -2289,7 +2289,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2328,7 +2328,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -2367,7 +2367,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2394,10 +2394,10 @@
         <v>736611</v>
       </c>
       <c r="I49" t="n">
-        <v>15050</v>
+        <v>21500</v>
       </c>
       <c r="J49" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K49" t="n">
         <v>21500</v>
@@ -2406,7 +2406,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -2445,7 +2445,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2507,7 +2507,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Steam 인기 차트 — 2026-09-12</t>
+          <t>Steam 인기 차트 — 2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3174,28 +3174,28 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="n">
+      <c r="A29" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Rust</t>
         </is>
       </c>
-      <c r="C29" t="n">
+      <c r="C29" s="4" t="n">
         <v>143870</v>
       </c>
-      <c r="D29" t="n">
+      <c r="D29" s="4" t="n">
         <v>87.2</v>
       </c>
-      <c r="E29" t="n">
+      <c r="E29" s="4" t="n">
         <v>1227784</v>
       </c>
-      <c r="F29" t="n">
-        <v>42000</v>
-      </c>
-      <c r="G29" t="n">
-        <v>0</v>
+      <c r="F29" s="4" t="n">
+        <v>21000</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="30">
@@ -3724,28 +3724,28 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="n">
+      <c r="A51" t="n">
         <v>48</v>
       </c>
-      <c r="B51" s="4" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>Phasmophobia</t>
         </is>
       </c>
-      <c r="C51" s="4" t="n">
+      <c r="C51" t="n">
         <v>9978</v>
       </c>
-      <c r="D51" s="4" t="n">
+      <c r="D51" t="n">
         <v>95.8</v>
       </c>
-      <c r="E51" s="4" t="n">
+      <c r="E51" t="n">
         <v>768779</v>
       </c>
-      <c r="F51" s="4" t="n">
-        <v>15050</v>
-      </c>
-      <c r="G51" s="4" t="n">
-        <v>30</v>
+      <c r="F51" t="n">
+        <v>21500</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -3830,7 +3830,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-09-12</t>
+          <t>2주(14일)+ 상위 50위 유지 게임 — 기준일: 2026-09-13</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3940,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-09-12</t>
+          <t>4주(28일)+ 상위 50위 유지 게임 — 기준일: 2026-09-13</t>
         </is>
       </c>
     </row>

</xml_diff>